<commit_message>
perf: updated PJS_levels with new variables in v2_sak_m_res
</commit_message>
<xml_diff>
--- a/data-raw/PJS_levels.xlsx
+++ b/data-raw/PJS_levels.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\13hopp\Documents\GitHub\NVIdb\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE016C1-D454-4BD7-9C46-0E44E551E2A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21405" windowHeight="8805"/>
+    <workbookView xWindow="3360" yWindow="75" windowWidth="21600" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ark1'!$A$1:$I$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ark1'!$A$1:$I$107</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
   <si>
     <t>aar</t>
   </si>
@@ -372,13 +373,43 @@
   </si>
   <si>
     <t>subres_operator</t>
+  </si>
+  <si>
+    <t>annen_aktor_rollekode</t>
+  </si>
+  <si>
+    <t>gatepostnr</t>
+  </si>
+  <si>
+    <t>vekt_volum</t>
+  </si>
+  <si>
+    <t>enhetstypekode</t>
+  </si>
+  <si>
+    <t>innsendelse_sist_endret</t>
+  </si>
+  <si>
+    <t>prove_sist_endret</t>
+  </si>
+  <si>
+    <t>delpr_sist_endret</t>
+  </si>
+  <si>
+    <t>und_sist_endret</t>
+  </si>
+  <si>
+    <t>res_sist_endret</t>
+  </si>
+  <si>
+    <t>konkl_sist_endret</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -390,6 +421,12 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Trebuchet MS"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -416,13 +453,13 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -702,1019 +739,1113 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I107"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I117"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="7" width="14.7109375" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="11.5703125" style="2"/>
+    <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>93</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2">
-        <v>1</v>
-      </c>
-      <c r="E2" s="4">
-        <v>1</v>
-      </c>
-      <c r="F2" s="4">
-        <v>1</v>
-      </c>
-      <c r="G2" s="4">
-        <v>1</v>
-      </c>
-      <c r="H2" s="4">
-        <v>1</v>
-      </c>
-      <c r="I2" s="4">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" s="3">
+        <v>1</v>
+      </c>
+      <c r="F2" s="3">
+        <v>1</v>
+      </c>
+      <c r="G2" s="3">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3">
+        <v>1</v>
+      </c>
+      <c r="I2" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2">
-        <v>1</v>
-      </c>
-      <c r="E3" s="4">
-        <v>1</v>
-      </c>
-      <c r="F3" s="4">
-        <v>1</v>
-      </c>
-      <c r="G3" s="4">
-        <v>1</v>
-      </c>
-      <c r="H3" s="4">
-        <v>1</v>
-      </c>
-      <c r="I3" s="4">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3">
+        <v>1</v>
+      </c>
+      <c r="F3" s="3">
+        <v>1</v>
+      </c>
+      <c r="G3" s="3">
+        <v>1</v>
+      </c>
+      <c r="H3" s="3">
+        <v>1</v>
+      </c>
+      <c r="I3" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2">
-        <v>1</v>
-      </c>
-      <c r="E4" s="4">
-        <v>1</v>
-      </c>
-      <c r="F4" s="4">
-        <v>1</v>
-      </c>
-      <c r="G4" s="4">
-        <v>1</v>
-      </c>
-      <c r="H4" s="4">
-        <v>1</v>
-      </c>
-      <c r="I4" s="4">
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3">
+        <v>1</v>
+      </c>
+      <c r="G4" s="3">
+        <v>1</v>
+      </c>
+      <c r="H4" s="3">
+        <v>1</v>
+      </c>
+      <c r="I4" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="2">
-        <v>1</v>
-      </c>
-      <c r="D5" s="2">
-        <v>1</v>
-      </c>
-      <c r="E5" s="4">
-        <v>1</v>
-      </c>
-      <c r="F5" s="4">
-        <v>1</v>
-      </c>
-      <c r="G5" s="4">
-        <v>1</v>
-      </c>
-      <c r="H5" s="4">
-        <v>1</v>
-      </c>
-      <c r="I5" s="4">
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1</v>
+      </c>
+      <c r="G5" s="3">
+        <v>1</v>
+      </c>
+      <c r="H5" s="3">
+        <v>1</v>
+      </c>
+      <c r="I5" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D6" s="2">
-        <v>1</v>
-      </c>
-      <c r="E6" s="4">
-        <v>1</v>
-      </c>
-      <c r="F6" s="4">
-        <v>1</v>
-      </c>
-      <c r="H6" s="4">
-        <v>1</v>
-      </c>
-      <c r="I6" s="4">
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3">
+        <v>1</v>
+      </c>
+      <c r="H6" s="3">
+        <v>1</v>
+      </c>
+      <c r="I6" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E7" s="4">
-        <v>1</v>
-      </c>
-      <c r="F7" s="4">
-        <v>1</v>
-      </c>
-      <c r="H7" s="4">
-        <v>1</v>
-      </c>
-      <c r="I7" s="4">
+      <c r="E7" s="3">
+        <v>1</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1</v>
+      </c>
+      <c r="H7" s="3">
+        <v>1</v>
+      </c>
+      <c r="I7" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4">
-        <v>1</v>
-      </c>
-      <c r="H8" s="4">
-        <v>1</v>
-      </c>
-      <c r="I8" s="4">
+      <c r="E8" s="3"/>
+      <c r="F8" s="3">
+        <v>1</v>
+      </c>
+      <c r="H8" s="3">
+        <v>1</v>
+      </c>
+      <c r="I8" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="2">
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="H10" s="4">
-        <v>1</v>
-      </c>
-      <c r="I10" s="4">
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="H10" s="3">
+        <v>1</v>
+      </c>
+      <c r="I10" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4">
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B23" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
+      <c r="B24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B24" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
+      <c r="B25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B25" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
+      <c r="B26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
+      <c r="B27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B27" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
+      <c r="B28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B28" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" s="4" t="s">
+      <c r="B29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B29" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
+      <c r="B30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B30" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" s="4" t="s">
+      <c r="B31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B31" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
+      <c r="B32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B32" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="4" t="s">
+      <c r="B33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B33" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="4" t="s">
+      <c r="B34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B34" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="4" t="s">
+      <c r="B35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B35" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="4" t="s">
+      <c r="B36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B36" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="4" t="s">
+      <c r="B37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B37" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="4" t="s">
+      <c r="B38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B38" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="4" t="s">
+      <c r="B39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B39" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="4" t="s">
+      <c r="B40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B40" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="4" t="s">
+      <c r="B41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B41" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="4" t="s">
+      <c r="B43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A44" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C42" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="4" t="s">
+      <c r="C45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C43" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="4" t="s">
+      <c r="C46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C44" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="4" t="s">
+      <c r="C47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C45" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="4" t="s">
+      <c r="C48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C46" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="4" t="s">
+      <c r="C49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C47" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="4" t="s">
+      <c r="C50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C48" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="4" t="s">
+      <c r="C51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C49" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="4" t="s">
+      <c r="C52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C50" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="4" t="s">
+      <c r="C53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C51" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" s="4" t="s">
+      <c r="C54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C52" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="4" t="s">
+      <c r="C55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C53" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="4" t="s">
+      <c r="C56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C54" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="4" t="s">
+      <c r="C57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A58" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A59" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C55" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56" s="4" t="s">
+      <c r="C60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C56" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="4" t="s">
+      <c r="C61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C57" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="4" t="s">
+      <c r="C62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C58" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="4" t="s">
+      <c r="C63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A64" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C59" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="4" t="s">
+      <c r="C64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C60" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="4" t="s">
+      <c r="C65">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C61" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="4" t="s">
+      <c r="C66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C62" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="4" t="s">
+      <c r="C67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C63" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="4" t="s">
+      <c r="C68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C64" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="4" t="s">
+      <c r="C69">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C65" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A66" s="4" t="s">
+      <c r="C70">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C66" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="4" t="s">
+      <c r="C71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C67" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A68" s="4" t="s">
+      <c r="C72">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C68" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="4" t="s">
+      <c r="C73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C69" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A70" s="4" t="s">
+      <c r="C74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C70" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="4" t="s">
+      <c r="C75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C71" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A72" s="4" t="s">
+      <c r="C76">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C72" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A73" s="4" t="s">
+      <c r="C77">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C73" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A74" s="4" t="s">
+      <c r="C78">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C74" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A75" s="4" t="s">
+      <c r="C79">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C75" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A76" s="4" t="s">
+      <c r="C80">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A81" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C76" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A77" s="4" t="s">
+      <c r="C81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A82" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C77" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A78" s="4" t="s">
+      <c r="C82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A83" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C78" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A79" s="4" t="s">
+      <c r="C83">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A84" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C79" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A80" s="4" t="s">
+      <c r="C84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A85" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C80" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A81" s="4" t="s">
+      <c r="C85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A86" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C81" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A82" s="4" t="s">
+      <c r="C86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A87" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C87">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A88" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D82" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A83" s="4" t="s">
+      <c r="D88">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A89" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D83" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A84" s="4" t="s">
+      <c r="D89">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A90" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D84" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A85" s="4" t="s">
+      <c r="D90">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A91" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D85" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A86" s="4" t="s">
+      <c r="D91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A92" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D86" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A87" s="4" t="s">
+      <c r="D92">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A93" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D87" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A88" s="4" t="s">
+      <c r="D93">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A94" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D94">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A95" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="E88" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A89" s="4" t="s">
+      <c r="E95">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A96" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="E89" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A90" s="4" t="s">
+      <c r="E96">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A97" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E90" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A91" s="4" t="s">
+      <c r="E97">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A98" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E98">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A99" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="F91" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A92" s="4" t="s">
+      <c r="F99">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A100" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="F92" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A93" s="4" t="s">
+      <c r="F100">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A101" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="F93" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A94" s="4" t="s">
+      <c r="F101">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A102" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F94" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A95" s="4" t="s">
+      <c r="F102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A103" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="F95" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A96" s="4" t="s">
+      <c r="F103">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A104" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="F104">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A105" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="G96" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A97" s="4" t="s">
+      <c r="G105">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A106" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="G97" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A98" s="4" t="s">
+      <c r="G106">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A107" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="G98" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A99" s="4" t="s">
+      <c r="G107">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A108" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="G108">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A109" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="H99" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A100" s="4" t="s">
+      <c r="H109">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A110" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="H100" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A101" s="4" t="s">
+      <c r="H110">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A111" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="H101" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A102" s="4" t="s">
+      <c r="H111">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A112" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="H102" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A103" s="4" t="s">
+      <c r="H112">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A113" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="I103" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A104" s="4" t="s">
+      <c r="I113">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A114" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="I104" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A105" s="4" t="s">
+      <c r="I114">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A115" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="I105" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A106" s="4" t="s">
+      <c r="I115">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A116" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="I106" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A107" s="2" t="s">
+      <c r="I116">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A117" t="s">
         <v>114</v>
       </c>
-      <c r="I107" s="2">
+      <c r="I117">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I98"/>
+  <autoFilter ref="A1:I107" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004E8DCD7061C9614189F6D0F57B1C8645" ma:contentTypeVersion="9" ma:contentTypeDescription="Opprett et nytt dokument." ma:contentTypeScope="" ma:versionID="d59b8845ebd1283ad3bf6a548e8d2471">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="077b9b9c-7f67-45a8-98b7-b654137cbace" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="972a228023c3d388b754ae5803fd6dc7" ns3:_="">
     <xsd:import namespace="077b9b9c-7f67-45a8-98b7-b654137cbace"/>
@@ -1892,22 +2023,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EAD5715D-3B45-4FFF-A267-1B867BA53632}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="077b9b9c-7f67-45a8-98b7-b654137cbace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D016577-9F2B-4060-8113-F67317A7ACDD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4347BC88-2E0B-468E-8A95-CF71CAD2677B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1923,28 +2063,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D016577-9F2B-4060-8113-F67317A7ACDD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EAD5715D-3B45-4FFF-A267-1B867BA53632}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="077b9b9c-7f67-45a8-98b7-b654137cbace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
perf: included variable anamnese in PJS_levels
</commit_message>
<xml_diff>
--- a/data-raw/PJS_levels.xlsx
+++ b/data-raw/PJS_levels.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\13hopp\Documents\GitHub\NVIdb\data-raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\13hopp\Documents\GitHub\NVIpjsr\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE016C1-D454-4BD7-9C46-0E44E551E2A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32721DF9-2C47-4644-880F-1A625029B619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3360" yWindow="75" windowWidth="21600" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ark1'!$A$1:$I$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ark1'!$A$1:$I$108</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="126">
   <si>
     <t>aar</t>
   </si>
@@ -403,6 +403,9 @@
   </si>
   <si>
     <t>konkl_sist_endret</t>
+  </si>
+  <si>
+    <t>anamnese</t>
   </si>
 </sst>
 </file>
@@ -740,7 +743,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I117"/>
+  <dimension ref="A1:I118"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
@@ -1231,25 +1234,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A44" s="4" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="B44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C45">
+      <c r="B45">
         <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C46">
         <v>1</v>
@@ -1257,7 +1260,7 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C47">
         <v>1</v>
@@ -1265,7 +1268,7 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C48">
         <v>1</v>
@@ -1273,7 +1276,7 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C49">
         <v>1</v>
@@ -1281,7 +1284,7 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -1289,7 +1292,7 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -1297,7 +1300,7 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -1305,7 +1308,7 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C53">
         <v>1</v>
@@ -1313,7 +1316,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C54">
         <v>1</v>
@@ -1321,7 +1324,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C55">
         <v>1</v>
@@ -1329,7 +1332,7 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C56">
         <v>1</v>
@@ -1337,15 +1340,15 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="C57">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A58" s="4" t="s">
-        <v>117</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -1353,15 +1356,15 @@
     </row>
     <row r="59" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A60" s="4" t="s">
         <v>118</v>
-      </c>
-      <c r="C59">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="3" t="s">
-        <v>46</v>
       </c>
       <c r="C60">
         <v>1</v>
@@ -1369,7 +1372,7 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C61">
         <v>1</v>
@@ -1377,7 +1380,7 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C62">
         <v>1</v>
@@ -1385,7 +1388,7 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C63">
         <v>1</v>
@@ -1393,7 +1396,7 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C64">
         <v>1</v>
@@ -1401,7 +1404,7 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C65">
         <v>1</v>
@@ -1409,7 +1412,7 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C66">
         <v>1</v>
@@ -1417,7 +1420,7 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C67">
         <v>1</v>
@@ -1425,7 +1428,7 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C68">
         <v>1</v>
@@ -1433,7 +1436,7 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C69">
         <v>1</v>
@@ -1441,7 +1444,7 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C70">
         <v>1</v>
@@ -1449,7 +1452,7 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C71">
         <v>1</v>
@@ -1457,7 +1460,7 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C72">
         <v>1</v>
@@ -1465,7 +1468,7 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C73">
         <v>1</v>
@@ -1473,7 +1476,7 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C74">
         <v>1</v>
@@ -1481,7 +1484,7 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C75">
         <v>1</v>
@@ -1489,7 +1492,7 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C76">
         <v>1</v>
@@ -1497,7 +1500,7 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C77">
         <v>1</v>
@@ -1505,7 +1508,7 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C78">
         <v>1</v>
@@ -1513,7 +1516,7 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C79">
         <v>1</v>
@@ -1521,7 +1524,7 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C80">
         <v>1</v>
@@ -1529,7 +1532,7 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C81">
         <v>1</v>
@@ -1537,7 +1540,7 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C82">
         <v>1</v>
@@ -1545,7 +1548,7 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C83">
         <v>1</v>
@@ -1553,7 +1556,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C84">
         <v>1</v>
@@ -1561,7 +1564,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C85">
         <v>1</v>
@@ -1569,31 +1572,31 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A87" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C86">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A87" s="4" t="s">
+      <c r="C87">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A88" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C87">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A88" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D88">
+      <c r="C88">
         <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D89">
         <v>1</v>
@@ -1601,7 +1604,7 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D90">
         <v>1</v>
@@ -1609,7 +1612,7 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D91">
         <v>1</v>
@@ -1617,7 +1620,7 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D92">
         <v>1</v>
@@ -1625,31 +1628,31 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D93">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A94" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D93">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A94" s="4" t="s">
+      <c r="D94">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A95" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="D94">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A95" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="E95">
+      <c r="D95">
         <v>1</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -1657,31 +1660,31 @@
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E97">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A98" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E97">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="98" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A98" s="4" t="s">
+      <c r="E98">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A99" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="E98">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A99" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F99">
+      <c r="E99">
         <v>1</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F100">
         <v>1</v>
@@ -1689,7 +1692,7 @@
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F101">
         <v>1</v>
@@ -1697,7 +1700,7 @@
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F102">
         <v>1</v>
@@ -1705,31 +1708,31 @@
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F103">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A104" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="F103">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="104" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A104" s="4" t="s">
+      <c r="F104">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A105" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="F104">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A105" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="G105">
+      <c r="F105">
         <v>1</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A106" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G106">
         <v>1</v>
@@ -1737,31 +1740,31 @@
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A107" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="G107">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A108" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="G107">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="108" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A108" s="4" t="s">
+      <c r="G108">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A109" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="G108">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A109" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="H109">
+      <c r="G109">
         <v>1</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A110" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H110">
         <v>1</v>
@@ -1769,7 +1772,7 @@
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A111" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H111">
         <v>1</v>
@@ -1777,7 +1780,7 @@
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A112" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H112">
         <v>1</v>
@@ -1785,15 +1788,15 @@
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A113" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="I113">
+        <v>109</v>
+      </c>
+      <c r="H113">
         <v>1</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A114" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I114">
         <v>1</v>
@@ -1801,7 +1804,7 @@
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I115">
         <v>1</v>
@@ -1809,43 +1812,36 @@
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A116" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="I116">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A117" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="I116">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A117" t="s">
+      <c r="I117">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A118" t="s">
         <v>114</v>
       </c>
-      <c r="I117">
+      <c r="I118">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I107" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:I108" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004E8DCD7061C9614189F6D0F57B1C8645" ma:contentTypeVersion="9" ma:contentTypeDescription="Opprett et nytt dokument." ma:contentTypeScope="" ma:versionID="d59b8845ebd1283ad3bf6a548e8d2471">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="077b9b9c-7f67-45a8-98b7-b654137cbace" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="972a228023c3d388b754ae5803fd6dc7" ns3:_="">
     <xsd:import namespace="077b9b9c-7f67-45a8-98b7-b654137cbace"/>
@@ -2023,31 +2019,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EAD5715D-3B45-4FFF-A267-1B867BA53632}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="077b9b9c-7f67-45a8-98b7-b654137cbace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D016577-9F2B-4060-8113-F67317A7ACDD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4347BC88-2E0B-468E-8A95-CF71CAD2677B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2063,4 +2050,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D016577-9F2B-4060-8113-F67317A7ACDD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EAD5715D-3B45-4FFF-A267-1B867BA53632}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="077b9b9c-7f67-45a8-98b7-b654137cbace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
perf: included uttatt2 in PJS_levels.xlsx
</commit_message>
<xml_diff>
--- a/data-raw/PJS_levels.xlsx
+++ b/data-raw/PJS_levels.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\13hopp\Documents\GitHub\NVIpjsr\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32721DF9-2C47-4644-880F-1A625029B619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D776262B-3FB1-4C19-BA77-72967BD62D42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ark1'!$A$1:$I$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ark1'!$A$1:$I$109</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="127">
   <si>
     <t>aar</t>
   </si>
@@ -406,6 +406,9 @@
   </si>
   <si>
     <t>anamnese</t>
+  </si>
+  <si>
+    <t>uttatt2</t>
   </si>
 </sst>
 </file>
@@ -743,7 +746,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I118"/>
+  <dimension ref="A1:I119"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
@@ -1036,7 +1039,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>10</v>
+        <v>126</v>
       </c>
       <c r="B19">
         <v>1</v>
@@ -1044,7 +1047,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B20">
         <v>1</v>
@@ -1052,7 +1055,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -1060,23 +1063,23 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
+      <c r="B23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
         <v>115</v>
-      </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
-        <v>14</v>
       </c>
       <c r="B24">
         <v>1</v>
@@ -1084,7 +1087,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B25">
         <v>1</v>
@@ -1092,7 +1095,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B26">
         <v>1</v>
@@ -1100,7 +1103,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B27">
         <v>1</v>
@@ -1108,7 +1111,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B28">
         <v>1</v>
@@ -1116,7 +1119,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B29">
         <v>1</v>
@@ -1124,7 +1127,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30">
         <v>1</v>
@@ -1132,7 +1135,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B31">
         <v>1</v>
@@ -1140,7 +1143,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B32">
         <v>1</v>
@@ -1148,7 +1151,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B33">
         <v>1</v>
@@ -1156,7 +1159,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B34">
         <v>1</v>
@@ -1164,7 +1167,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B35">
         <v>1</v>
@@ -1172,7 +1175,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B36">
         <v>1</v>
@@ -1180,7 +1183,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B37">
         <v>1</v>
@@ -1188,7 +1191,7 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B38">
         <v>1</v>
@@ -1196,7 +1199,7 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B39">
         <v>1</v>
@@ -1204,7 +1207,7 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
-        <v>100</v>
+        <v>29</v>
       </c>
       <c r="B40">
         <v>1</v>
@@ -1212,7 +1215,7 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="B41">
         <v>1</v>
@@ -1220,7 +1223,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
-        <v>116</v>
+        <v>30</v>
       </c>
       <c r="B42">
         <v>1</v>
@@ -1228,7 +1231,7 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
-        <v>31</v>
+        <v>116</v>
       </c>
       <c r="B43">
         <v>1</v>
@@ -1236,31 +1239,31 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A45" s="4" t="s">
+      <c r="B45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="B45">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C46">
+      <c r="B46">
         <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C47">
         <v>1</v>
@@ -1268,7 +1271,7 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C48">
         <v>1</v>
@@ -1276,7 +1279,7 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C49">
         <v>1</v>
@@ -1284,7 +1287,7 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -1292,7 +1295,7 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -1300,7 +1303,7 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -1308,7 +1311,7 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C53">
         <v>1</v>
@@ -1316,7 +1319,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C54">
         <v>1</v>
@@ -1324,7 +1327,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C55">
         <v>1</v>
@@ -1332,7 +1335,7 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C56">
         <v>1</v>
@@ -1340,7 +1343,7 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C57">
         <v>1</v>
@@ -1348,15 +1351,15 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="C58">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A59" s="4" t="s">
-        <v>117</v>
       </c>
       <c r="C59">
         <v>1</v>
@@ -1364,15 +1367,15 @@
     </row>
     <row r="60" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A61" s="4" t="s">
         <v>118</v>
-      </c>
-      <c r="C60">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="3" t="s">
-        <v>46</v>
       </c>
       <c r="C61">
         <v>1</v>
@@ -1380,7 +1383,7 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C62">
         <v>1</v>
@@ -1388,7 +1391,7 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C63">
         <v>1</v>
@@ -1396,7 +1399,7 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C64">
         <v>1</v>
@@ -1404,7 +1407,7 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C65">
         <v>1</v>
@@ -1412,7 +1415,7 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C66">
         <v>1</v>
@@ -1420,7 +1423,7 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C67">
         <v>1</v>
@@ -1428,7 +1431,7 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C68">
         <v>1</v>
@@ -1436,7 +1439,7 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C69">
         <v>1</v>
@@ -1444,7 +1447,7 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C70">
         <v>1</v>
@@ -1452,7 +1455,7 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C71">
         <v>1</v>
@@ -1460,7 +1463,7 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C72">
         <v>1</v>
@@ -1468,7 +1471,7 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C73">
         <v>1</v>
@@ -1476,7 +1479,7 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C74">
         <v>1</v>
@@ -1484,7 +1487,7 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C75">
         <v>1</v>
@@ -1492,7 +1495,7 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C76">
         <v>1</v>
@@ -1500,7 +1503,7 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C77">
         <v>1</v>
@@ -1508,7 +1511,7 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C78">
         <v>1</v>
@@ -1516,7 +1519,7 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C79">
         <v>1</v>
@@ -1524,143 +1527,143 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C80">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A81" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C80">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A81" s="3" t="s">
+      <c r="C81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A82" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C81">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A82" s="3" t="s">
+      <c r="C82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A83" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C82">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A83" s="3" t="s">
+      <c r="C83">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A84" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C83">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A84" s="3" t="s">
+      <c r="C84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A85" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C84">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A85" s="3" t="s">
+      <c r="C85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A86" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C85">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A86" s="3" t="s">
+      <c r="C86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A87" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C86">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A87" s="3" t="s">
+      <c r="C87">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A88" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C87">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A88" s="4" t="s">
+      <c r="C88">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A89" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C88">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A89" s="3" t="s">
+      <c r="C89">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A90" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D89">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A90" s="3" t="s">
+      <c r="D90">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A91" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D90">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A91" s="3" t="s">
+      <c r="D91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A92" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D91">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A92" s="3" t="s">
+      <c r="D92">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A93" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D92">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A93" s="3" t="s">
+      <c r="D93">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A94" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D93">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A94" s="3" t="s">
+      <c r="D94">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A95" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D94">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A95" s="4" t="s">
+      <c r="D95">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A96" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="D95">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A96" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="E96">
+      <c r="D96">
         <v>1</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -1668,31 +1671,31 @@
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E98">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A99" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E98">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="99" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A99" s="4" t="s">
+      <c r="E99">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A100" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="E99">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A100" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F100">
+      <c r="E100">
         <v>1</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F101">
         <v>1</v>
@@ -1700,7 +1703,7 @@
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F102">
         <v>1</v>
@@ -1708,7 +1711,7 @@
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F103">
         <v>1</v>
@@ -1716,31 +1719,31 @@
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A104" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F104">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A105" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="F104">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="105" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A105" s="4" t="s">
+      <c r="F105">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A106" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="F105">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A106" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="G106">
+      <c r="F106">
         <v>1</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A107" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G107">
         <v>1</v>
@@ -1748,31 +1751,31 @@
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A108" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="G108">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A109" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="G108">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="109" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A109" s="4" t="s">
+      <c r="G109">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A110" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="G109">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A110" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="H110">
+      <c r="G110">
         <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A111" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H111">
         <v>1</v>
@@ -1780,7 +1783,7 @@
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A112" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H112">
         <v>1</v>
@@ -1788,7 +1791,7 @@
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A113" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H113">
         <v>1</v>
@@ -1796,15 +1799,15 @@
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A114" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="I114">
+        <v>109</v>
+      </c>
+      <c r="H114">
         <v>1</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I115">
         <v>1</v>
@@ -1812,7 +1815,7 @@
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A116" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I116">
         <v>1</v>
@@ -1820,28 +1823,51 @@
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A117" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="I117">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A118" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="I117">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A118" t="s">
+      <c r="I118">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
         <v>114</v>
       </c>
-      <c r="I118">
+      <c r="I119">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I108" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:I109" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004E8DCD7061C9614189F6D0F57B1C8645" ma:contentTypeVersion="9" ma:contentTypeDescription="Opprett et nytt dokument." ma:contentTypeScope="" ma:versionID="d59b8845ebd1283ad3bf6a548e8d2471">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="077b9b9c-7f67-45a8-98b7-b654137cbace" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="972a228023c3d388b754ae5803fd6dc7" ns3:_="">
     <xsd:import namespace="077b9b9c-7f67-45a8-98b7-b654137cbace"/>
@@ -2019,22 +2045,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EAD5715D-3B45-4FFF-A267-1B867BA53632}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="077b9b9c-7f67-45a8-98b7-b654137cbace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D016577-9F2B-4060-8113-F67317A7ACDD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4347BC88-2E0B-468E-8A95-CF71CAD2677B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2050,28 +2085,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D016577-9F2B-4060-8113-F67317A7ACDD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EAD5715D-3B45-4FFF-A267-1B867BA53632}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="077b9b9c-7f67-45a8-98b7-b654137cbace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>